<commit_message>
add display_name to shelves table
</commit_message>
<xml_diff>
--- a/new_seed/demo-scenario.xlsx
+++ b/new_seed/demo-scenario.xlsx
@@ -1797,7 +1797,7 @@
         <v>BOX-H-20260701-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>A-01-01</v>
+        <v>A0101</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1814,7 +1814,7 @@
         <v>BOX-H-20260701-0002</v>
       </c>
       <c r="B3" t="str">
-        <v>A-01-02</v>
+        <v>A0102</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -1831,7 +1831,7 @@
         <v>BOX-H-20260701-0003</v>
       </c>
       <c r="B4" t="str">
-        <v>A-02-01</v>
+        <v>A0201</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1848,7 +1848,7 @@
         <v>BOX-H-20260701-0004</v>
       </c>
       <c r="B5" t="str">
-        <v>A-02-02</v>
+        <v>A0202</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -1865,7 +1865,7 @@
         <v>BOX-H-20260701-0005</v>
       </c>
       <c r="B6" t="str">
-        <v>A-03-01</v>
+        <v>A0301</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1882,7 +1882,7 @@
         <v>BOX-H-20260701-0006</v>
       </c>
       <c r="B7" t="str">
-        <v>A-03-02</v>
+        <v>A0302</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -1899,7 +1899,7 @@
         <v>BOX-H-20260701-0007</v>
       </c>
       <c r="B8" t="str">
-        <v>A-03-03</v>
+        <v>A0303</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -1916,7 +1916,7 @@
         <v>BOX-H-20260701-0008</v>
       </c>
       <c r="B9" t="str">
-        <v>A-03-04</v>
+        <v>A0304</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -1933,7 +1933,7 @@
         <v>BOX-H-20260701-0009</v>
       </c>
       <c r="B10" t="str">
-        <v>A-03-05</v>
+        <v>A0305</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1950,7 +1950,7 @@
         <v>BOX-H-20260701-0010</v>
       </c>
       <c r="B11" t="str">
-        <v>A-04-01</v>
+        <v>A0401</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -1967,7 +1967,7 @@
         <v>BOX-H-20260701-0011</v>
       </c>
       <c r="B12" t="str">
-        <v>A-04-02</v>
+        <v>A0402</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1984,7 +1984,7 @@
         <v>BOX-H-20260701-0012</v>
       </c>
       <c r="B13" t="str">
-        <v>A-04-03</v>
+        <v>A0403</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -2001,7 +2001,7 @@
         <v>BOX-H-20260701-0013</v>
       </c>
       <c r="B14" t="str">
-        <v>A-04-04</v>
+        <v>A0404</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -2018,7 +2018,7 @@
         <v>BOX-H-20260701-0014</v>
       </c>
       <c r="B15" t="str">
-        <v>A-04-05</v>
+        <v>A0405</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -2072,7 +2072,7 @@
         <v>BOX-H-20260701-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>A-01-01</v>
+        <v>A0101</v>
       </c>
       <c r="C2" t="str">
         <v>RK73H1JTTD1002F</v>
@@ -2098,7 +2098,7 @@
         <v>BOX-H-20260701-0001</v>
       </c>
       <c r="B3" t="str">
-        <v>A-01-01</v>
+        <v>A0101</v>
       </c>
       <c r="C3" t="str">
         <v>RK73H1JTTD2202F</v>
@@ -2124,7 +2124,7 @@
         <v>BOX-H-20260701-0002</v>
       </c>
       <c r="B4" t="str">
-        <v>A-01-02</v>
+        <v>A0102</v>
       </c>
       <c r="C4" t="str">
         <v>RK73B1JTTD181G</v>
@@ -2150,7 +2150,7 @@
         <v>BOX-H-20260701-0002</v>
       </c>
       <c r="B5" t="str">
-        <v>A-01-02</v>
+        <v>A0102</v>
       </c>
       <c r="C5" t="str">
         <v>RK73H1JTTD4702F</v>
@@ -2176,7 +2176,7 @@
         <v>BOX-H-20260701-0003</v>
       </c>
       <c r="B6" t="str">
-        <v>A-02-01</v>
+        <v>A0201</v>
       </c>
       <c r="C6" t="str">
         <v>RK73H1JTTD5602F</v>
@@ -2202,7 +2202,7 @@
         <v>BOX-H-20260701-0003</v>
       </c>
       <c r="B7" t="str">
-        <v>A-02-01</v>
+        <v>A0201</v>
       </c>
       <c r="C7" t="str">
         <v>RK73H2ATTD2212F</v>
@@ -2366,7 +2366,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>A-03-01..A-04-05 — print their labels with apps/web's</v>
+        <v>A0301..A0405 — print their labels with apps/web's</v>
       </c>
     </row>
     <row r="28">

</xml_diff>